<commit_message>
docs: confirm P0-2 G-3 finalized in coverage matrix (2026-09-02 Final Gate)
</commit_message>
<xml_diff>
--- a/docs/asset/coverage-matrix-summary.xlsx
+++ b/docs/asset/coverage-matrix-summary.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2592" uniqueCount="1401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2592" uniqueCount="1402">
   <si>
     <t>引用文档一览</t>
   </si>
@@ -3894,6 +3894,9 @@
     <t>本ブックの母体資料</t>
   </si>
   <si>
+    <t>✅ 完了（2026-09-02・G-3 確定）</t>
+  </si>
+  <si>
     <t>サーバ縦断ループ</t>
   </si>
   <si>
@@ -3996,7 +3999,7 @@
     <t>連字符有無が口徑差</t>
   </si>
   <si>
-    <t>✅ G-3 暫定判定済（2026-09-02・Final Gate 確認待ち）</t>
+    <t>✅ G-1〜G-3 通過（2026-09-02・G-3 確定）</t>
   </si>
   <si>
     <t>文書 ID 台帳（IDR-01 §2.1/§3 出典）</t>
@@ -8070,7 +8073,7 @@
         <v>1278</v>
       </c>
       <c r="F33" t="s">
-        <v>1276</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -8078,19 +8081,19 @@
         <v>261</v>
       </c>
       <c r="B34" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="C34" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="D34" t="s">
+        <v>1282</v>
+      </c>
+      <c r="E34" t="s">
+        <v>1283</v>
+      </c>
+      <c r="F34" t="s">
         <v>1281</v>
-      </c>
-      <c r="E34" t="s">
-        <v>1282</v>
-      </c>
-      <c r="F34" t="s">
-        <v>1280</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -8098,39 +8101,39 @@
         <v>253</v>
       </c>
       <c r="B35" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="C35" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="D35" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="E35" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="F35" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
       <c r="B36" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="C36" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="D36" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="E36" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="F36" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -8138,24 +8141,24 @@
         <v>366</v>
       </c>
       <c r="B37" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="C37" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="D37" t="s">
+        <v>1293</v>
+      </c>
+      <c r="E37" t="s">
+        <v>1294</v>
+      </c>
+      <c r="F37" t="s">
         <v>1292</v>
-      </c>
-      <c r="E37" t="s">
-        <v>1293</v>
-      </c>
-      <c r="F37" t="s">
-        <v>1291</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="22" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="B39" s="23"/>
       <c r="C39" s="23"/>
@@ -8167,16 +8170,16 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="B40" t="s">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="C40" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="F40" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="G40" t="s">
         <v>269</v>
@@ -8184,13 +8187,13 @@
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="B41" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="F41" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="G41" t="s">
         <v>269</v>
@@ -8198,16 +8201,16 @@
     </row>
     <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
       <c r="B42" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="C42" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="F42" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="G42" t="s">
         <v>323</v>
@@ -8215,30 +8218,30 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="B43" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="F43" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="G43" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="B44" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="C44" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="F44" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="G44" t="s">
         <v>269</v>
@@ -8266,12 +8269,12 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" spans="1:4">
       <c r="A1" s="19" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="20" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -8279,10 +8282,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="D3" s="21" t="s">
         <v>159</v>
@@ -8296,10 +8299,10 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="D4" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -8310,10 +8313,10 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
+        <v>1321</v>
+      </c>
+      <c r="D5" t="s">
         <v>1320</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1319</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -8324,24 +8327,24 @@
         <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="D6" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="B7" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="C7" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="D7" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -8352,10 +8355,10 @@
         <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="D8" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -8366,24 +8369,24 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="D9" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="B10" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="C10" t="s">
         <v>82</v>
       </c>
       <c r="D10" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -8394,10 +8397,10 @@
         <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="D11" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -8408,10 +8411,10 @@
         <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="D12" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -8422,24 +8425,24 @@
         <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="D13" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="B14" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="C14" t="s">
         <v>82</v>
       </c>
       <c r="D14" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -8450,10 +8453,10 @@
         <v>46</v>
       </c>
       <c r="C15" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="D15" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -8464,38 +8467,38 @@
         <v>50</v>
       </c>
       <c r="C16" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="D16" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="B17" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="C17" t="s">
         <v>82</v>
       </c>
       <c r="D17" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B18" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="C18" t="s">
         <v>82</v>
       </c>
       <c r="D18" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -8506,10 +8509,10 @@
         <v>54</v>
       </c>
       <c r="C19" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="D19" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -8520,24 +8523,24 @@
         <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="D20" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="B21" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="C21" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="D21" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -8548,66 +8551,66 @@
         <v>63</v>
       </c>
       <c r="C22" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="D22" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B23" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="C23" t="s">
         <v>82</v>
       </c>
       <c r="D23" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="B24" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="C24" t="s">
         <v>82</v>
       </c>
       <c r="D24" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="B25" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="C25" t="s">
         <v>82</v>
       </c>
       <c r="D25" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="B26" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="C26" t="s">
         <v>82</v>
       </c>
       <c r="D26" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -8618,10 +8621,10 @@
         <v>67</v>
       </c>
       <c r="C27" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="D27" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -8632,10 +8635,10 @@
         <v>79</v>
       </c>
       <c r="C28" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="D28" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -8646,10 +8649,10 @@
         <v>75</v>
       </c>
       <c r="C29" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="D29" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -8660,10 +8663,10 @@
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="D30" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -8674,10 +8677,10 @@
         <v>70</v>
       </c>
       <c r="C31" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="D31" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -8685,13 +8688,13 @@
         <v>69</v>
       </c>
       <c r="B32" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="C32" t="s">
         <v>82</v>
       </c>
       <c r="D32" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -8699,13 +8702,13 @@
         <v>69</v>
       </c>
       <c r="B33" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="C33" t="s">
         <v>82</v>
       </c>
       <c r="D33" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -8716,10 +8719,10 @@
         <v>72</v>
       </c>
       <c r="C34" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="D34" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -8727,13 +8730,13 @@
         <v>69</v>
       </c>
       <c r="B35" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="C35" t="s">
         <v>82</v>
       </c>
       <c r="D35" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -8741,13 +8744,13 @@
         <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="C36" t="s">
         <v>82</v>
       </c>
       <c r="D36" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -8755,13 +8758,13 @@
         <v>69</v>
       </c>
       <c r="B37" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="C37" t="s">
         <v>82</v>
       </c>
       <c r="D37" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -8769,13 +8772,13 @@
         <v>69</v>
       </c>
       <c r="B38" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="C38" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="D38" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -8783,13 +8786,13 @@
         <v>69</v>
       </c>
       <c r="B39" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="C39" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="D39" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
   </sheetData>
@@ -8816,17 +8819,17 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:64">
       <c r="A1" s="1" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:64">
       <c r="A2" s="2" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:64">
       <c r="A3" s="3" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="B3" s="15" t="str">
         <f>IF('3.機能一覧'!A4="","",'3.機能一覧'!A4)</f>
@@ -9069,7 +9072,7 @@
         <v/>
       </c>
       <c r="BJ3" s="9" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="BK3" s="9" t="s">
         <v>157</v>
@@ -9085,7 +9088,7 @@
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
@@ -9164,7 +9167,7 @@
         <v>REQ-002</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -9246,7 +9249,7 @@
       <c r="B6" s="5"/>
       <c r="C6" s="6"/>
       <c r="D6" s="6" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -9327,7 +9330,7 @@
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -9408,7 +9411,7 @@
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
@@ -9489,7 +9492,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="6" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -9570,7 +9573,7 @@
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="6"/>
@@ -9651,7 +9654,7 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="J11" s="5"/>
       <c r="K11" s="6"/>
@@ -9732,7 +9735,7 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
@@ -9813,7 +9816,7 @@
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
@@ -9894,7 +9897,7 @@
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
       <c r="L14" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
@@ -9976,7 +9979,7 @@
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
       <c r="N15" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="O15" s="5"/>
       <c r="P15" s="5"/>
@@ -10055,7 +10058,7 @@
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
       <c r="M16" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
@@ -10124,43 +10127,43 @@
         <v>REQ-014</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="O17" s="5"/>
       <c r="P17" s="5"/>
@@ -10241,7 +10244,7 @@
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
       <c r="O18" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="P18" s="5"/>
       <c r="Q18" s="5"/>
@@ -10325,7 +10328,7 @@
       <c r="Q19" s="5"/>
       <c r="R19" s="5"/>
       <c r="S19" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="T19" s="5"/>
       <c r="U19" s="5"/>
@@ -10404,7 +10407,7 @@
       <c r="P20" s="5"/>
       <c r="Q20" s="5"/>
       <c r="R20" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="S20" s="5"/>
       <c r="T20" s="5"/>
@@ -10483,7 +10486,7 @@
       <c r="O21" s="5"/>
       <c r="P21" s="5"/>
       <c r="Q21" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="R21" s="5"/>
       <c r="S21" s="5"/>
@@ -10563,7 +10566,7 @@
       <c r="O22" s="5"/>
       <c r="P22" s="5"/>
       <c r="Q22" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="R22" s="5"/>
       <c r="S22" s="5"/>
@@ -10646,7 +10649,7 @@
       <c r="R23" s="5"/>
       <c r="S23" s="5"/>
       <c r="T23" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="U23" s="5"/>
       <c r="V23" s="5"/>
@@ -10727,7 +10730,7 @@
       <c r="S24" s="5"/>
       <c r="T24" s="5"/>
       <c r="U24" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="V24" s="5"/>
       <c r="W24" s="5"/>
@@ -10808,7 +10811,7 @@
       <c r="T25" s="5"/>
       <c r="U25" s="5"/>
       <c r="V25" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W25" s="5"/>
       <c r="X25" s="5"/>
@@ -10888,7 +10891,7 @@
       <c r="T26" s="5"/>
       <c r="U26" s="5"/>
       <c r="V26" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W26" s="5"/>
       <c r="X26" s="5"/>
@@ -10963,17 +10966,17 @@
       <c r="O27" s="5"/>
       <c r="P27" s="5"/>
       <c r="Q27" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="R27" s="5"/>
       <c r="S27" s="5"/>
       <c r="T27" s="5"/>
       <c r="U27" s="5"/>
       <c r="V27" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W27" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="X27" s="5"/>
       <c r="Y27" s="5"/>
@@ -11053,7 +11056,7 @@
       <c r="U28" s="5"/>
       <c r="V28" s="5"/>
       <c r="W28" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="X28" s="5"/>
       <c r="Y28" s="5"/>
@@ -11128,13 +11131,13 @@
       <c r="P29" s="5"/>
       <c r="Q29" s="5"/>
       <c r="R29" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="S29" s="5"/>
       <c r="T29" s="5"/>
       <c r="U29" s="5"/>
       <c r="V29" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W29" s="5"/>
       <c r="X29" s="5"/>
@@ -11214,7 +11217,7 @@
       <c r="T30" s="5"/>
       <c r="U30" s="5"/>
       <c r="V30" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W30" s="5"/>
       <c r="X30" s="5"/>
@@ -11294,7 +11297,7 @@
       <c r="T31" s="5"/>
       <c r="U31" s="5"/>
       <c r="V31" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W31" s="5"/>
       <c r="X31" s="5"/>
@@ -11369,14 +11372,14 @@
       <c r="O32" s="5"/>
       <c r="P32" s="5"/>
       <c r="Q32" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="R32" s="5"/>
       <c r="S32" s="5"/>
       <c r="T32" s="5"/>
       <c r="U32" s="5"/>
       <c r="V32" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W32" s="5"/>
       <c r="X32" s="5"/>
@@ -11454,17 +11457,17 @@
       <c r="R33" s="5"/>
       <c r="S33" s="5"/>
       <c r="T33" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="U33" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="V33" s="5"/>
       <c r="W33" s="5"/>
       <c r="X33" s="5"/>
       <c r="Y33" s="5"/>
       <c r="Z33" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="AA33" s="5"/>
       <c r="AB33" s="5"/>
@@ -11540,7 +11543,7 @@
       <c r="T34" s="5"/>
       <c r="U34" s="5"/>
       <c r="V34" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W34" s="5"/>
       <c r="X34" s="5"/>
@@ -11693,7 +11696,7 @@
       <c r="O36" s="5"/>
       <c r="P36" s="5"/>
       <c r="Q36" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="R36" s="5"/>
       <c r="S36" s="5"/>
@@ -11705,7 +11708,7 @@
       <c r="Y36" s="5"/>
       <c r="Z36" s="5"/>
       <c r="AA36" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="AB36" s="5"/>
       <c r="AC36" s="5"/>
@@ -11782,7 +11785,7 @@
       <c r="V37" s="5"/>
       <c r="W37" s="5"/>
       <c r="X37" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="Y37" s="5"/>
       <c r="Z37" s="5"/>
@@ -12021,7 +12024,7 @@
       <c r="Y40" s="5"/>
       <c r="Z40" s="5"/>
       <c r="AA40" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="AB40" s="5"/>
       <c r="AC40" s="5"/>
@@ -12099,7 +12102,7 @@
       <c r="W41" s="5"/>
       <c r="X41" s="5"/>
       <c r="Y41" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="Z41" s="5"/>
       <c r="AA41" s="5"/>
@@ -12331,10 +12334,10 @@
       <c r="S44" s="5"/>
       <c r="T44" s="5"/>
       <c r="U44" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="V44" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W44" s="5"/>
       <c r="X44" s="5"/>
@@ -12799,25 +12802,25 @@
       <c r="O50" s="5"/>
       <c r="P50" s="5"/>
       <c r="Q50" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="R50" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="S50" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="T50" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="U50" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="V50" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="W50" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="X50" s="5"/>
       <c r="Y50" s="5"/>
@@ -13526,7 +13529,7 @@
     </row>
     <row r="64" ht="33" customHeight="1" spans="1:64">
       <c r="A64" s="9" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="B64" s="17">
         <f t="shared" ref="B64:BI64" si="4">IF(B$3="","",SUMPRODUCT(($A$4:$A$63&lt;&gt;"")*(B$4:B$63="○")))</f>
@@ -14069,17 +14072,17 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:84">
       <c r="A1" s="1" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:84">
       <c r="A2" s="2" t="s">
-        <v>1377</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:84">
       <c r="A3" s="3" t="s">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="B3" s="15" t="str">
         <f>IF('4.画面一覧'!A4="","",'4.画面一覧'!A4)</f>
@@ -14402,7 +14405,7 @@
         <v/>
       </c>
       <c r="CD3" s="9" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="CE3" s="9" t="s">
         <v>157</v>
@@ -14417,7 +14420,7 @@
         <v>F-01</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
@@ -14518,7 +14521,7 @@
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
@@ -14717,7 +14720,7 @@
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
@@ -14817,7 +14820,7 @@
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -14917,7 +14920,7 @@
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
@@ -15017,7 +15020,7 @@
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
@@ -15117,7 +15120,7 @@
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
@@ -15217,7 +15220,7 @@
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
@@ -15318,7 +15321,7 @@
       <c r="C13" s="6"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
@@ -15418,7 +15421,7 @@
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
@@ -15518,7 +15521,7 @@
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
@@ -15618,7 +15621,7 @@
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
@@ -15719,7 +15722,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="5"/>
@@ -16014,7 +16017,7 @@
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
@@ -16116,7 +16119,7 @@
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
@@ -16217,7 +16220,7 @@
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
       <c r="H22" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
@@ -16317,7 +16320,7 @@
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
       <c r="H23" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
@@ -16515,7 +16518,7 @@
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
       <c r="H25" s="5" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
@@ -20329,7 +20332,7 @@
     </row>
     <row r="64" ht="33" customHeight="1" spans="1:84">
       <c r="A64" s="9" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
       <c r="B64" s="17">
         <f t="shared" ref="B64:BM64" si="1">IF(B$3="","",SUMPRODUCT(($A$4:$A$63&lt;&gt;"")*(B$4:B$63="○")))</f>
@@ -21000,37 +21003,37 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7">
       <c r="A2" s="2" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:7">
       <c r="B4" s="3" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>157</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:7">
       <c r="B5" s="4" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="C5" s="5">
         <f>COUNTA('2.要件一覧'!$A$4:$A$63)</f>
@@ -21049,12 +21052,12 @@
         <v>⚠ 要対応</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:7">
       <c r="B6" s="4" t="s">
-        <v>1389</v>
+        <v>1390</v>
       </c>
       <c r="C6" s="5">
         <f>COUNTA('3.機能一覧'!$A$4:$A$63)</f>
@@ -21073,12 +21076,12 @@
         <v>⚠ 要対応</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>1390</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:7">
       <c r="B7" s="4" t="s">
-        <v>1391</v>
+        <v>1392</v>
       </c>
       <c r="C7" s="5">
         <f>COUNTA('3.機能一覧'!$A$4:$A$63)</f>
@@ -21097,12 +21100,12 @@
         <v>⚠ 要対応</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>1392</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:7">
       <c r="B8" s="4" t="s">
-        <v>1393</v>
+        <v>1394</v>
       </c>
       <c r="C8" s="5">
         <f>COUNTA('4.画面一覧'!$A$4:$A$83)</f>
@@ -21121,12 +21124,12 @@
         <v>OK</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>1394</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:7">
       <c r="B10" s="9" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
       <c r="C10" s="10" t="str">
         <f>IF(SUM($D$5:$D$8)=0,"✅ 全て割当済み（缺口 0 件）","⚠ 未割当 "&amp;SUM($D$5:$D$8)&amp;" 件あり — 去 2〜4 各表看橙色行")</f>
@@ -21139,12 +21142,12 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:7">
       <c r="B12" s="13" t="s">
-        <v>1396</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:7">
       <c r="B13" s="4" t="s">
-        <v>1397</v>
+        <v>1398</v>
       </c>
       <c r="C13" s="14">
         <f>'14.要件×機能行列'!$BJ$64</f>
@@ -21153,7 +21156,7 @@
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:7">
       <c r="B14" s="4" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="C14" s="14">
         <f>'15.機能×画面行列'!$CD$64</f>
@@ -21162,7 +21165,7 @@
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:7">
       <c r="B15" s="4" t="s">
-        <v>1399</v>
+        <v>1400</v>
       </c>
       <c r="C15" s="14">
         <f>IFERROR('14.要件×機能行列'!$BJ$64/$C$5,"-")</f>
@@ -21171,7 +21174,7 @@
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:7">
       <c r="B16" s="4" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="C16" s="14">
         <f>IFERROR('15.機能×画面行列'!$CD$64/$C$6,"-")</f>

</xml_diff>

<commit_message>
docs: sync P0-3 implementation status (D-4 writeback + S-3 partial-implementation alignment)
</commit_message>
<xml_diff>
--- a/docs/asset/coverage-matrix-summary.xlsx
+++ b/docs/asset/coverage-matrix-summary.xlsx
@@ -2505,7 +2505,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>未実施（P0-3 計画）</t>
+          <t>✅ 実施済（2026-09-02・S-3/T-1・BookingProjectionRestTest 15/15 PASS）</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>未実施（P0-3 計画）</t>
+          <t>✅ 実施済（2026-09-02・S-3/T-1・BookingProjectionRestTest 15/15 PASS）</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>未実施（P0-3 計画）</t>
+          <t>✅ 実施済（2026-09-02・S-3/T-1・BookingProjectionRestTest 15/15 PASS）</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>未実施（P0-3 計画）</t>
+          <t>✅ 実施済（2026-09-02・S-3/T-1・BookingProjectionRestTest 15/15 PASS）</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>未実施（P0-3 計画）</t>
+          <t>✅ 実施済（2026-09-02・S-3/T-1・BookingProjectionRestTest 15/15 PASS）</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>未実施（P0-3 計画）</t>
+          <t>✅ 実施済（2026-09-02・S-3/T-1・BookingProjectionRestTest 15/15 PASS）</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3685,7 +3685,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -4293,7 +4292,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="22" t="inlineStr">
         <is>
@@ -4574,7 +4572,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -4710,7 +4707,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>対応計画済・未着手（P0-2〜P0-4）</t>
+          <t>部分対応（監査フィールド設置済〔P0-2 S-1/S-2〕・記録実装は P0-3 残）</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4742,7 +4739,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>対応計画済・未着手（P0-2〜P0-4）</t>
+          <t>部分対応（方針凍結済〔RULE-11・CHK-01 C-2・2026-09-01〕）</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4806,7 +4803,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>対応計画済・未着手（P0-2〜P0-4）</t>
+          <t>部分対応（設計確定〔CHK-02 C-3〕＋行級制御設置済〔P0-2 S-3/S-4〕・runtime 実装は P0-3 残）</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4838,7 +4835,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>部分対応（P0 手動 Retry・残り P1）</t>
+          <t>対応計画済・未着手（P0-3 計画〔REQ-027/028・S-4/B-7 未実装〕・残り P1）</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4879,7 +4876,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="22" t="inlineStr">
         <is>
@@ -5020,7 +5016,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>未決（P0-3 NC 設定前）</t>
+          <t>✅ 決定済（2026-09-02・CHK-02 C-1＝booking-deploy 公網 HTTPS）</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -5167,7 +5163,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="22" t="inlineStr">
         <is>
@@ -5243,7 +5238,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="22" t="inlineStr">
         <is>
@@ -5369,7 +5363,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>🔵 進行中</t>
+          <t>✅ 完了（2026-09-02・G-3 確定）</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -5401,7 +5395,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>⬜ 未着手</t>
+          <t>🔵 進行中（SF 側 S-1〜S-3 済〔11a7c78/907fe02/6b9d970〕・S-4/S-5/B 系 残）</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -5416,7 +5410,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>⬜ 未着手</t>
+          <t>🔵 進行中（SF 側 S-1〜S-3 済・S-4/S-5/T-2〜T-5 残）</t>
         </is>
       </c>
     </row>
@@ -5516,7 +5510,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="22" t="inlineStr">
         <is>
@@ -18918,7 +18911,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -19063,7 +19055,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="B10" s="9" t="inlineStr">
         <is>
@@ -19079,7 +19070,6 @@
       <c r="F10" s="11" t="n"/>
       <c r="G10" s="12" t="n"/>
     </row>
-    <row r="11"/>
     <row r="12" ht="15" customHeight="1">
       <c r="B12" s="13" t="inlineStr">
         <is>
@@ -19158,7 +19148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -19181,7 +19171,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -19335,7 +19324,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1">
       <c r="B14" s="13" t="inlineStr">
         <is>
@@ -19403,7 +19391,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="15" customHeight="1">
       <c r="B21" s="13" t="inlineStr">
         <is>
@@ -19443,7 +19430,6 @@
       </c>
       <c r="C25" s="12" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
@@ -19553,6 +19539,13 @@
       <c r="A42" t="inlineStr">
         <is>
           <t>【2026-09-02 P0-2 実施完了反映】B-1〜B-3・S-1〜S-5 実施済（12.F41/F42・71c88c8・aec1bf4/f020618/bc7a4ac）・G-1〜G-3 通過（G-3 暫定判定・12.F44）・REQ-030/031 部分実施（2.G33/K33・G34/K34）・CD-06/07/08・TERM 系 実装/設置反映（8・7）・IDR-01 V1.4（引用文档一览 E4）・CHK-01 V1.7/PPT-01 V1.5 追従</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>【2026-09-03 回写反映】監査発見の文書遅延分を回写：REQ-018/024/029/030/031 部分実施（P0-3 SF 側 S-1〜S-3 実装〔11a7c78/907fe02/6b9d970〕）・F-20 部分実施・P0-2 工程行 C 列完了統一・G3 決定済反映。連動版数：RD-01 V1.2・BD-02 V2.1・DD-01 V1.1・PPT-01 V1.6・CHK-02 V1.7（D-4 実行・REQ-021 文案修正）</t>
         </is>
       </c>
     </row>
@@ -20395,7 +20388,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>ユーザー管理：ユーザー作成・照会・状態変更（セッション取消）・ロール変更（セッション維持）・削除</t>
+          <t>ユーザー管理：ユーザー作成・照会・状態変更（セッション取消）・ロール変更（旧トークン拒否）・削除</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -20720,7 +20713,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>未着手（P0-3 計画）</t>
+          <t>部分実施（SF 側受入口 BookingProjectionRest 済〔6b9d970〕・Booking 側呼出残）</t>
         </is>
       </c>
       <c r="H21" s="5">
@@ -20738,7 +20731,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>🔵 P0-3 計画</t>
+          <t>🔵 部分実施（SF 側受入口済〔6b9d970〕・Booking 側残）</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -21080,7 +21073,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>部分実施（schema migration 済・runtime P0-3）</t>
+          <t>部分実施（schema migration 済〔71c88c8〕＋SF runtime 版本ゲート済〔VR・6b9d970〕・Booking runtime 残）</t>
         </is>
       </c>
       <c r="H27" s="5">
@@ -21098,7 +21091,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>🔵 部分実施（schema 済・P0-3 残）</t>
+          <t>🔵 部分実施（schema＋SF runtime 済・Booking 残）</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -21380,7 +21373,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>未着手（P0-3 計画）</t>
+          <t>部分実施（SF 側 A2/A3 設備済〔ECA/NC/EC・2026-09-02〕・MV-11 検証未実施）</t>
         </is>
       </c>
       <c r="H32" s="5">
@@ -21398,7 +21391,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>🔵 P0-3 計画</t>
+          <t>🔵 部分実施（SF 側設備済・検証残）</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -23353,7 +23346,7 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>状態遷移検証（RULE-05・RULE-07）のうえ変更・取消を実施。取消確認メールは非同期送信。ハード削除あり</t>
+          <t>状態遷移検証（RULE-05・RULE-07）のうえ変更・取消を実施。取消確認メールは非同期送信。DELETE は取消動作（status→CANCELLED・行保留）</t>
         </is>
       </c>
       <c r="D11" s="24" t="inlineStr">
@@ -23589,7 +23582,7 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>ユーザー作成・照会・統計、状態変更（セッション取消）、ロール変更（セッション維持＝現行仕様・既知課題）、削除</t>
+          <t>ユーザー作成・照会・統計、状態変更（セッション取消）、ロール変更（旧トークン拒否・guard 化済・DB セッション行対応は P1）、削除</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -23862,7 +23855,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>🔵 P0-3 計画</t>
+          <t>🔵 部分実施（SF 側受入口済〔6b9d970〕・Booking 側残）</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -28247,7 +28240,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ユーザー状態変更は全セッション取消。ロール変更はセッション維持（現行仕様・既知課題）</t>
+          <t>ユーザー状態変更は全セッション取消。ロール変更は既存セッション行を残すが guard 化により旧トークンは拒否（DB セッション行対応は P1）</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -29458,7 +29451,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -29581,7 +29573,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="22" t="inlineStr">
         <is>
@@ -30012,7 +30003,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="22" t="inlineStr">
         <is>
@@ -30320,7 +30310,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="22" t="inlineStr">
         <is>

</xml_diff>